<commit_message>
Media batch 11: import and frame-by-frame QC (9 of 24 clips pass)
12 first-workout exercises in both sexes from the Flow project
"out. 04 - 05:39". Pass: band_overhead_press f/m, band_pull_apart f/m,
cable_woodchop f/m, band_lat_pulldown f, bridge_floor_press f,
cable_chest_fly m. The other 15 are listed in qc.json with the defect
(no pull on the assisted pull-up, hip thrust done as a seated squat,
Pallof done as a fly, both legs together in the dead bug, white glows,
short ranges). Raw files removed; videos.js, media-redo, the launch-set
sheet and lists rebuilt (3 more exercises now have clips for both sexes).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YZKDqVTirwP3vm8p6KZMpS
</commit_message>
<xml_diff>
--- a/docs/review/launch-set.xlsx
+++ b/docs/review/launch-set.xlsx
@@ -11403,7 +11403,7 @@
       </c>
       <c r="E130" s="8" t="inlineStr">
         <is>
-          <t>missing (coming)</t>
+          <t>band_lat_pulldown.f.mp4</t>
         </is>
       </c>
       <c r="F130" s="8" t="inlineStr">
@@ -11488,12 +11488,12 @@
       </c>
       <c r="E131" s="8" t="inlineStr">
         <is>
-          <t>missing (coming)</t>
+          <t>band_overhead_press.f.mp4</t>
         </is>
       </c>
       <c r="F131" s="8" t="inlineStr">
         <is>
-          <t>missing (coming)</t>
+          <t>band_overhead_press.m.mp4</t>
         </is>
       </c>
       <c r="G131" s="8" t="inlineStr">
@@ -11574,12 +11574,12 @@
       </c>
       <c r="E132" s="8" t="inlineStr">
         <is>
-          <t>missing (coming)</t>
+          <t>band_pull_apart.f.mp4</t>
         </is>
       </c>
       <c r="F132" s="8" t="inlineStr">
         <is>
-          <t>missing (coming)</t>
+          <t>band_pull_apart.m.mp4</t>
         </is>
       </c>
       <c r="G132" s="8" t="inlineStr">
@@ -11820,7 +11820,7 @@
       </c>
       <c r="E135" s="8" t="inlineStr">
         <is>
-          <t>missing (coming)</t>
+          <t>bridge_floor_press.f.mp4</t>
         </is>
       </c>
       <c r="F135" s="8" t="inlineStr">
@@ -11995,7 +11995,7 @@
       </c>
       <c r="F137" s="8" t="inlineStr">
         <is>
-          <t>missing (coming)</t>
+          <t>cable_chest_fly.m.mp4</t>
         </is>
       </c>
       <c r="G137" s="8" t="inlineStr">
@@ -12154,12 +12154,12 @@
       </c>
       <c r="E139" s="8" t="inlineStr">
         <is>
-          <t>missing (coming)</t>
+          <t>cable_woodchop.f.mp4</t>
         </is>
       </c>
       <c r="F139" s="8" t="inlineStr">
         <is>
-          <t>missing (coming)</t>
+          <t>cable_woodchop.m.mp4</t>
         </is>
       </c>
       <c r="G139" s="8" t="inlineStr">

</xml_diff>

<commit_message>
Phase 32 A: shoulder safety
- Shoulder program exercise 11 is now the dumbbell triceps kickback (AAOS),
  replacing the overhead triceps extension.
- Nothing above 90 degrees or behind the back while the shoulder program runs
  or with shoulder pain: read from the database joint tags, enforced in the
  program sessions, in the generator (shoulderCap) and in the swap sheet,
  including inside a program session. Stretch 3 (behind the back) is left out.
- The physio question has "Yes / No / Not sure", nothing pre-selected; the
  strengthening (sessions B and C, the daily blocks) opens only on "Yes".
- "Full dose" and "Strengthening before the workout" start off (store v3
  resets them); switches are teal when on and selected chips show a check.
- Launch set, reviewer sheet and Flow lists regenerated (kickback in).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YZKDqVTirwP3vm8p6KZMpS
</commit_message>
<xml_diff>
--- a/docs/review/launch-set.xlsx
+++ b/docs/review/launch-set.xlsx
@@ -20292,12 +20292,12 @@
       </c>
       <c r="B237" s="8" t="inlineStr">
         <is>
-          <t>overhead_dumbbell_triceps_extension</t>
+          <t>dumbbell_kickback</t>
         </is>
       </c>
       <c r="C237" s="8" t="inlineStr">
         <is>
-          <t>Overhead triceps extension</t>
+          <t>Dumbbell triceps kickback</t>
         </is>
       </c>
       <c r="D237" s="8" t="inlineStr">
@@ -20317,12 +20317,13 @@
       </c>
       <c r="G237" s="8" t="inlineStr">
         <is>
-          <t>Triceps (Triceps brachii): primary, 1.0</t>
+          <t>Triceps (Triceps brachii): primary, 1.0
+Rear shoulders (Deltoid · rear head): secondary, 0.2</t>
         </is>
       </c>
       <c r="H237" s="8" t="inlineStr">
         <is>
-          <t>Dumbbells</t>
+          <t>Dumbbells, Flat bench</t>
         </is>
       </c>
       <c r="I237" s="8" t="inlineStr">
@@ -20331,7 +20332,7 @@
         </is>
       </c>
       <c r="J237" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K237" s="8" t="inlineStr">
         <is>
@@ -20340,17 +20341,17 @@
       </c>
       <c r="L237" s="8" t="inlineStr">
         <is>
-          <t>Standing, Seated</t>
+          <t>Standing, With support</t>
         </is>
       </c>
       <c r="M237" s="8" t="inlineStr">
         <is>
-          <t>Shoulder, Elbow / wrist</t>
+          <t>Elbow / wrist, Recent surgery</t>
         </is>
       </c>
       <c r="N237" s="8" t="inlineStr">
         <is>
-          <t>Hold a dumbbell overhead; lower behind your head and extend.</t>
+          <t>One hand on the bench, upper arm along your side, straighten the elbow back and squeeze.</t>
         </is>
       </c>
       <c r="O237" s="8" t="inlineStr">
@@ -20360,10 +20361,9 @@
       </c>
       <c r="P237" s="8" t="inlineStr">
         <is>
-          <t>Shoulder: Arm overhead (full)
-Elbow: Straighten elbow with weight (full)
-Elbow: Bend elbow with weight (full)
-Wrist: Grip tight (full)</t>
+          <t>Elbow: Straighten elbow with weight (full)
+Shoulder: Pull (hold, no movement)
+Wrist: Grip tight (partial)</t>
         </is>
       </c>
       <c r="Q237" s="9" t="n"/>

</xml_diff>